<commit_message>
docs: add design system reference specifications
Define configuration structures for Google, LibreOffice, Material, Microsoft 365, and WPS design systems to guide UI/UX development.
</commit_message>
<xml_diff>
--- a/tests/cellina/Sample-1.xlsx
+++ b/tests/cellina/Sample-1.xlsx
@@ -1,36 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{32958EAC-80FB-764F-97F6-B15F3C960ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Database" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sort 1" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Sort 2" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Filter 1" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Filter 2" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Filter 3" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Advanced 1" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Advanced 2" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Advanced 3" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Rekapitulasi" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="Hasil Rekap" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="Subtotal" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Database" sheetId="1" r:id="rId1"/>
+    <sheet name="Sort 1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sort 2" sheetId="3" r:id="rId3"/>
+    <sheet name="Filter 1" sheetId="4" r:id="rId4"/>
+    <sheet name="Filter 2" sheetId="5" r:id="rId5"/>
+    <sheet name="Filter 3" sheetId="6" r:id="rId6"/>
+    <sheet name="Advanced 1" sheetId="7" r:id="rId7"/>
+    <sheet name="Advanced 2" sheetId="8" r:id="rId8"/>
+    <sheet name="Advanced 3" sheetId="9" r:id="rId9"/>
+    <sheet name="Rekapitulasi" sheetId="10" r:id="rId10"/>
+    <sheet name="Hasil Rekap" sheetId="11" r:id="rId11"/>
+    <sheet name="Subtotal" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Filter 1'!$A$4:$E$26</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Filter 2'!$A$4:$E$26</definedName>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Filter 3'!$A$4:$E$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Filter 1'!$A$4:$E$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Filter 2'!$A$4:$E$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Filter 3'!$A$4:$E$26</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId16"/>
+    <pivotCache cacheId="0" r:id="rId13"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
@@ -39,170 +50,151 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="45">
   <si>
-    <t xml:space="preserve">Data Pendaftar</t>
+    <t>Data Pendaftar</t>
   </si>
   <si>
-    <t xml:space="preserve">SMA N 2 Kota Sorong</t>
+    <t>SMA N 2 Kota Sorong</t>
   </si>
   <si>
-    <t xml:space="preserve">Tanggal Daftar</t>
+    <t>Tanggal Daftar</t>
   </si>
   <si>
-    <t xml:space="preserve">Nama</t>
+    <t>Nama</t>
   </si>
   <si>
-    <t xml:space="preserve">Asal Sekolah</t>
+    <t>Asal Sekolah</t>
   </si>
   <si>
-    <t xml:space="preserve">Jenis Kelamin</t>
+    <t>Jenis Kelamin</t>
   </si>
   <si>
-    <t xml:space="preserve">Nilai UASDA</t>
+    <t>Nilai UASDA</t>
   </si>
   <si>
-    <t xml:space="preserve">6 Juli 2006</t>
+    <t>6 Juli 2006</t>
   </si>
   <si>
-    <t xml:space="preserve">Eko Sulistyo</t>
+    <t>Eko Sulistyo</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Negeri 4</t>
+    <t>SMP Negeri 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Laki-laki</t>
+    <t>Laki-laki</t>
   </si>
   <si>
-    <t xml:space="preserve">Wulandari</t>
+    <t>Wulandari</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Negeri 2</t>
+    <t>SMP Negeri 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Perempuan</t>
+    <t>Perempuan</t>
   </si>
   <si>
-    <t xml:space="preserve">Budiman</t>
+    <t>Budiman</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Muhammadiyah 2</t>
+    <t>SMP Muhammadiyah 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Indriyani</t>
+    <t>Indriyani</t>
   </si>
   <si>
-    <t xml:space="preserve">Untung</t>
+    <t>Untung</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Negeri 9</t>
+    <t>SMP Negeri 9</t>
   </si>
   <si>
-    <t xml:space="preserve">Zumarnis</t>
+    <t>Zumarnis</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Muhammadiyah 1</t>
+    <t>SMP Muhammadiyah 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Khairullah</t>
+    <t>Khairullah</t>
   </si>
   <si>
-    <t xml:space="preserve">7 Juli 2006</t>
+    <t>7 Juli 2006</t>
   </si>
   <si>
-    <t xml:space="preserve">Diana</t>
+    <t>Diana</t>
   </si>
   <si>
-    <t xml:space="preserve">Kumaladewi</t>
+    <t>Kumaladewi</t>
   </si>
   <si>
-    <t xml:space="preserve">Qomarudin</t>
+    <t>Qomarudin</t>
   </si>
   <si>
-    <t xml:space="preserve">Firmansyah</t>
+    <t>Firmansyah</t>
   </si>
   <si>
-    <t xml:space="preserve">Hermini</t>
+    <t>Hermini</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Negeri 3</t>
+    <t>SMP Negeri 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Dewi Sandra</t>
+    <t>Dewi Sandra</t>
   </si>
   <si>
-    <t xml:space="preserve">Mulatno</t>
+    <t>Mulatno</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Negeri 1</t>
+    <t>SMP Negeri 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Liana</t>
+    <t>Liana</t>
   </si>
   <si>
-    <t xml:space="preserve">8 Juli 2006</t>
+    <t>8 Juli 2006</t>
   </si>
   <si>
-    <t xml:space="preserve">Purnomo</t>
+    <t>Purnomo</t>
   </si>
   <si>
-    <t xml:space="preserve">Sinta</t>
+    <t>Sinta</t>
   </si>
   <si>
-    <t xml:space="preserve">SMP Negeri 6</t>
+    <t>SMP Negeri 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Andriani</t>
+    <t>Andriani</t>
   </si>
   <si>
-    <t xml:space="preserve">Tanti</t>
+    <t>Tanti</t>
   </si>
   <si>
-    <t xml:space="preserve">Hartanto</t>
+    <t>Hartanto</t>
   </si>
   <si>
-    <t xml:space="preserve">Kurniawati</t>
+    <t>Kurniawati</t>
   </si>
   <si>
-    <t xml:space="preserve">Sartono</t>
+    <t>Sartono</t>
   </si>
   <si>
-    <t xml:space="preserve">Count of Asal Sekolah</t>
+    <t>Count of Asal Sekolah</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Result</t>
+    <t>Total Result</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.00"/>
-  </numFmts>
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="12"/>
@@ -212,7 +204,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Aptos Display"/>
@@ -220,7 +212,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FFFFFF00"/>
       <name val="Arial"/>
@@ -235,7 +227,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -264,317 +256,236 @@
     </fill>
   </fills>
   <borders count="15">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="34">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB3B3B3"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE6E6E6"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -633,25 +544,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="22" createdVersion="3">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedDate="0" createdVersion="3" recordCount="22" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A4:E26" sheet="Rekapitulasi"/>
   </cacheSource>
@@ -730,6 +645,11 @@
       </sharedItems>
     </cacheField>
   </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
 </pivotCacheDefinition>
 </file>
 
@@ -893,7 +813,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot table 1" cacheId="1" dataOnRows="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" showDrill="1" useAutoFormatting="0" itemPrintTitles="1" indent="0" outline="0" outlineData="0" compact="0" compactData="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0C00-000000000000}" name="Pivot table 1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" itemPrintTitles="1" indent="0" compact="0" compactData="0">
   <location ref="A1:D11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField showAll="0"/>
@@ -967,14 +887,19 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of Asal Sekolah" fld="2" subtotal="count" numFmtId="164"/>
+    <dataField name="Count of Asal Sekolah" fld="2" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleDark1" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
 </pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1016,14 +941,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="SimSun" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Times New Roman" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="SimSun"/>
+        <a:cs typeface="Times New Roman"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1053,7 +978,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1077,7 +1002,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1131,7 +1056,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1151,48 +1076,47 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1209,7 +1133,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -1226,7 +1150,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -1243,7 +1167,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -1260,7 +1184,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -1277,7 +1201,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -1294,7 +1218,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -1311,7 +1235,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -1328,7 +1252,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -1345,7 +1269,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -1362,7 +1286,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -1379,7 +1303,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -1396,7 +1320,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -1413,7 +1337,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -1430,7 +1354,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -1447,7 +1371,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -1464,7 +1388,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -1481,7 +1405,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -1498,7 +1422,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -1515,7 +1439,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -1532,7 +1456,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -1549,7 +1473,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -1566,7 +1490,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -1588,50 +1512,42 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1648,7 +1564,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -1665,7 +1581,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -1682,7 +1598,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -1699,7 +1615,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -1716,7 +1632,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -1733,7 +1649,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -1750,7 +1666,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -1767,7 +1683,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -1784,7 +1700,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -1801,7 +1717,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -1818,7 +1734,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -1835,7 +1751,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -1852,7 +1768,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -1869,7 +1785,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -1886,7 +1802,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -1903,7 +1819,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -1920,7 +1836,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -1937,7 +1853,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -1954,7 +1870,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -1971,7 +1887,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -1988,7 +1904,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -2005,7 +1921,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -2027,30 +1943,22 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="21.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="11.19"/>
+    <col min="1" max="1" width="21.3046875" style="12" customWidth="1"/>
+    <col min="2" max="2" width="16.046875" customWidth="1"/>
+    <col min="3" max="4" width="11.19140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A1" s="13" t="s">
         <v>42</v>
       </c>
@@ -2060,7 +1968,7 @@
       <c r="C1" s="15"/>
       <c r="D1" s="16"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A2" s="14" t="s">
         <v>4</v>
       </c>
@@ -2074,7 +1982,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A3" s="20" t="s">
         <v>20</v>
       </c>
@@ -2086,7 +1994,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A4" s="24" t="s">
         <v>15</v>
       </c>
@@ -2098,7 +2006,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A5" s="24" t="s">
         <v>31</v>
       </c>
@@ -2110,7 +2018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A6" s="24" t="s">
         <v>12</v>
       </c>
@@ -2124,7 +2032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A7" s="24" t="s">
         <v>28</v>
       </c>
@@ -2136,7 +2044,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A8" s="24" t="s">
         <v>9</v>
       </c>
@@ -2150,7 +2058,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A9" s="24" t="s">
         <v>36</v>
       </c>
@@ -2162,7 +2070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A10" s="24" t="s">
         <v>18</v>
       </c>
@@ -2176,7 +2084,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" ht="12.75" x14ac:dyDescent="0.15">
       <c r="A11" s="19" t="s">
         <v>43</v>
       </c>
@@ -2191,50 +2099,42 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2251,7 +2151,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -2268,7 +2168,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -2285,7 +2185,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -2302,7 +2202,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -2319,7 +2219,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -2336,7 +2236,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -2353,7 +2253,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
@@ -2370,7 +2270,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>33</v>
       </c>
@@ -2387,7 +2287,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>7</v>
       </c>
@@ -2404,7 +2304,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -2421,7 +2321,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>33</v>
       </c>
@@ -2438,7 +2338,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2455,7 +2355,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>33</v>
       </c>
@@ -2472,7 +2372,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>7</v>
       </c>
@@ -2489,7 +2389,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>7</v>
       </c>
@@ -2506,7 +2406,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>7</v>
       </c>
@@ -2523,7 +2423,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
@@ -2540,7 +2440,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -2557,7 +2457,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -2574,7 +2474,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>7</v>
       </c>
@@ -2591,7 +2491,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>22</v>
       </c>
@@ -2608,7 +2508,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -2630,50 +2530,42 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2690,7 +2582,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>33</v>
       </c>
@@ -2707,7 +2599,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -2724,7 +2616,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -2741,7 +2633,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -2758,7 +2650,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -2775,7 +2667,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -2792,7 +2684,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
@@ -2809,7 +2701,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -2826,7 +2718,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>7</v>
       </c>
@@ -2843,7 +2735,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
@@ -2860,7 +2752,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -2877,7 +2769,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>33</v>
       </c>
@@ -2894,7 +2786,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -2911,7 +2803,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -2928,7 +2820,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>33</v>
       </c>
@@ -2945,7 +2837,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
@@ -2962,7 +2854,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>33</v>
       </c>
@@ -2979,7 +2871,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -2996,7 +2888,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -3013,7 +2905,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>7</v>
       </c>
@@ -3030,7 +2922,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>7</v>
       </c>
@@ -3047,7 +2939,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>7</v>
       </c>
@@ -3069,50 +2961,42 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3129,7 +3013,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -3146,7 +3030,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -3163,7 +3047,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -3180,7 +3064,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>33</v>
       </c>
@@ -3197,7 +3081,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -3214,7 +3098,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>33</v>
       </c>
@@ -3231,7 +3115,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
@@ -3248,7 +3132,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>33</v>
       </c>
@@ -3265,7 +3149,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -3282,7 +3166,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
@@ -3299,7 +3183,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>33</v>
       </c>
@@ -3316,7 +3200,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -3333,7 +3217,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>33</v>
       </c>
@@ -3350,7 +3234,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>7</v>
       </c>
@@ -3367,7 +3251,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -3384,7 +3268,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>7</v>
       </c>
@@ -3401,7 +3285,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
@@ -3418,7 +3302,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -3435,7 +3319,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>7</v>
       </c>
@@ -3452,7 +3336,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>7</v>
       </c>
@@ -3469,7 +3353,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -3486,7 +3370,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>7</v>
       </c>
@@ -3508,50 +3392,43 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3568,7 +3445,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -3585,7 +3462,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -3602,7 +3479,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -3619,7 +3496,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -3636,7 +3513,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -3653,7 +3530,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -3670,7 +3547,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -3687,7 +3564,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -3704,7 +3581,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -3721,7 +3598,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -3738,7 +3615,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -3755,7 +3632,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -3772,7 +3649,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -3789,7 +3666,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -3806,7 +3683,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -3823,7 +3700,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -3840,7 +3717,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -3857,7 +3734,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -3874,7 +3751,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -3891,7 +3768,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -3908,7 +3785,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -3925,7 +3802,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -3943,7 +3820,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E26">
+  <autoFilter ref="A4:E26" xr:uid="{00000000-0009-0000-0000-000003000000}">
     <filterColumn colId="2">
       <filters>
         <filter val="SMP Negeri 4"/>
@@ -3954,51 +3831,43 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -4015,7 +3884,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -4032,7 +3901,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -4049,7 +3918,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -4066,7 +3935,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -4083,7 +3952,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -4100,7 +3969,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -4117,7 +3986,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -4134,7 +4003,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -4151,7 +4020,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -4168,7 +4037,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -4185,7 +4054,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -4202,7 +4071,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -4219,7 +4088,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -4236,7 +4105,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -4253,7 +4122,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -4270,7 +4139,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -4287,7 +4156,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -4304,7 +4173,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -4321,7 +4190,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -4338,7 +4207,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -4355,7 +4224,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -4372,7 +4241,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -4390,7 +4259,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E26">
+  <autoFilter ref="A4:E26" xr:uid="{00000000-0009-0000-0000-000004000000}">
     <filterColumn colId="2">
       <filters>
         <filter val="SMP Negeri 2"/>
@@ -4402,51 +4271,43 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -4463,7 +4324,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -4480,7 +4341,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -4497,7 +4358,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -4514,7 +4375,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -4531,7 +4392,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -4548,7 +4409,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -4565,7 +4426,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -4582,7 +4443,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -4599,7 +4460,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -4616,7 +4477,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -4633,7 +4494,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -4650,7 +4511,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -4667,7 +4528,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -4684,7 +4545,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -4701,7 +4562,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -4718,7 +4579,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -4735,7 +4596,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -4752,7 +4613,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -4769,7 +4630,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -4786,7 +4647,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -4803,7 +4664,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -4820,7 +4681,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -4838,63 +4699,54 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E26">
+  <autoFilter ref="A4:E26" xr:uid="{00000000-0009-0000-0000-000005000000}">
     <filterColumn colId="4">
-      <top10 top="true" percent="false" val="7"/>
+      <top10 val="7"/>
     </filterColumn>
   </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="9.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.55"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.9765625" style="2"/>
+    <col min="8" max="8" width="11.19140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.55078125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -4926,7 +4778,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -4958,7 +4810,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -4990,7 +4842,7 @@
         <v>25.9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -5022,7 +4874,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -5054,7 +4906,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -5086,7 +4938,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -5118,7 +4970,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -5150,7 +5002,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -5182,7 +5034,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -5214,7 +5066,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -5246,7 +5098,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -5278,7 +5130,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -5295,7 +5147,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -5312,7 +5164,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -5329,7 +5181,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -5346,7 +5198,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -5363,7 +5215,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -5380,7 +5232,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -5397,7 +5249,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -5414,7 +5266,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -5431,7 +5283,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -5448,7 +5300,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -5470,53 +5322,45 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="9.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.55"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.9765625" style="2"/>
+    <col min="8" max="8" width="11.19140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.55078125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -5548,7 +5392,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -5580,7 +5424,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -5612,7 +5456,7 @@
         <v>27.67</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -5644,7 +5488,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -5676,7 +5520,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -5708,7 +5552,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -5740,7 +5584,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -5772,7 +5616,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -5804,7 +5648,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -5836,7 +5680,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -5868,7 +5712,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -5900,7 +5744,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -5932,7 +5776,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -5964,7 +5808,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -5996,7 +5840,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -6013,7 +5857,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -6030,7 +5874,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -6047,7 +5891,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -6064,7 +5908,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -6081,7 +5925,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -6098,7 +5942,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -6115,7 +5959,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -6137,53 +5981,45 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.9765625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.73"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="9.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.55"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="9.97"/>
+    <col min="1" max="1" width="10.3828125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.5390625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.11328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.9765625" style="2"/>
+    <col min="8" max="8" width="11.19140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.55078125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9.9765625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -6215,7 +6051,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
@@ -6247,7 +6083,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
@@ -6279,7 +6115,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -6311,7 +6147,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -6343,7 +6179,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -6375,7 +6211,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -6407,7 +6243,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -6424,7 +6260,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -6441,7 +6277,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -6458,7 +6294,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -6475,7 +6311,7 @@
         <v>26.45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -6492,7 +6328,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -6509,7 +6345,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -6526,7 +6362,7 @@
         <v>27.85</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -6543,7 +6379,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -6560,7 +6396,7 @@
         <v>26.78</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>33</v>
       </c>
@@ -6577,7 +6413,7 @@
         <v>25.65</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
@@ -6594,7 +6430,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>33</v>
       </c>
@@ -6611,7 +6447,7 @@
         <v>27.92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
@@ -6628,7 +6464,7 @@
         <v>28.3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>33</v>
       </c>
@@ -6645,7 +6481,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
@@ -6662,7 +6498,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>33</v>
       </c>
@@ -6684,12 +6520,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="overThenDown" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>